<commit_message>
Mise à jour automatique
</commit_message>
<xml_diff>
--- a/articles.xlsx
+++ b/articles.xlsx
@@ -33,9 +33,6 @@
     <t>Le Mexique lance sa Coupe du Monde</t>
   </si>
   <si>
-    <t>le mexique lance parfaitement.html</t>
-  </si>
-  <si>
     <t>Denis prend la tête du championnat</t>
   </si>
   <si>
@@ -46,6 +43,9 @@
   </si>
   <si>
     <t>Présentation du tournoi</t>
+  </si>
+  <si>
+    <t>le mexique lance parfaitement son mondial.html</t>
   </si>
 </sst>
 </file>
@@ -388,7 +388,8 @@
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -405,7 +406,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="75">
+    <row r="2" spans="1:4" ht="60">
       <c r="A2" s="1">
         <v>46185</v>
       </c>
@@ -413,10 +414,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="60">
@@ -424,13 +425,13 @@
         <v>46184</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>